<commit_message>
Phase 129: History backend — TinyDB store with atomic writes and corrupt-file recovery, /api/history CRUD with search/filter/sort/pagination, auto-save of successful predictions, Insights aggregates; F16 draws the History store apart from the computing routes
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/00_evidence_index/evidence_index.xlsx
+++ b/outputs/00_evidence_index/evidence_index.xlsx
@@ -13245,12 +13245,12 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>F16</t>
+          <t>ALG-01</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O1, O6</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
@@ -13258,27 +13258,27 @@
       <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Dashboard system architecture</t>
+          <t>Dataset loading and master metadata construction</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/F16_dashboard_system_architecture.png</t>
+          <t>outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.txt</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>src/reporting/diagrams/pipeline_figures.py</t>
+          <t>src/data_loader/catalog.py; src/data_loader/circor.py; src/data_loader/duplicates.py; src/data_loader/integrity.py; src/data_loader/master.py; src/data_loader/pascal.py; src/data_loader/physionet.py</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>python scripts/05_render_diagrams.py --only F16</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-01</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>2026-09-11T18:19:31.153233+00:00</t>
+          <t>2026-09-11T18:56:56.769734+00:00</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -13288,19 +13288,19 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 7 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>ALG-01</t>
+          <t>ALG-02</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>O1, O6</t>
+          <t>O4</t>
         </is>
       </c>
       <c r="C243" t="inlineStr"/>
@@ -13308,27 +13308,27 @@
       <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Dataset loading and master metadata construction</t>
+          <t>Signal harmonization and resampling</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.txt</t>
+          <t>outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.txt</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>src/data_loader/catalog.py; src/data_loader/circor.py; src/data_loader/duplicates.py; src/data_loader/integrity.py; src/data_loader/master.py; src/data_loader/pascal.py; src/data_loader/physionet.py</t>
+          <t>src/preprocessing/io.py; src/preprocessing/pipeline.py; src/preprocessing/quality.py</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-01</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-02</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>2026-09-11T18:56:56.769734+00:00</t>
+          <t>2026-09-11T18:56:56.907550+00:00</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -13338,14 +13338,14 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>file and 7 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>ALG-02</t>
+          <t>ALG-03</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -13358,27 +13358,27 @@
       <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Signal harmonization and resampling</t>
+          <t>Butterworth filtering and z-score normalization</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.txt</t>
+          <t>outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.txt</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>src/preprocessing/io.py; src/preprocessing/pipeline.py; src/preprocessing/quality.py</t>
+          <t>src/preprocessing/filters.py; src/preprocessing/normalize.py</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-02</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-03</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>2026-09-11T18:56:56.907550+00:00</t>
+          <t>2026-09-11T18:56:59.243899+00:00</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -13388,14 +13388,14 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>ALG-03</t>
+          <t>ALG-04</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -13408,27 +13408,27 @@
       <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Butterworth filtering and z-score normalization</t>
+          <t>Multi-domain 138-feature extraction</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.txt</t>
+          <t>outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>src/preprocessing/filters.py; src/preprocessing/normalize.py</t>
+          <t>src/feature_extraction/extractor.py; src/feature_extraction/registry.py</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-03</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-04</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>2026-09-11T18:56:59.243899+00:00</t>
+          <t>2026-09-11T18:56:59.379027+00:00</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -13445,12 +13445,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>ALG-04</t>
+          <t>ALG-05</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -13458,27 +13458,27 @@
       <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Multi-domain 138-feature extraction</t>
+          <t>Fold-safe scaling and preprocessing</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt</t>
+          <t>outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.txt</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>src/feature_extraction/extractor.py; src/feature_extraction/registry.py</t>
+          <t>src/data_loader/splits.py; src/models/pipeline.py</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-04</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-05</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>2026-09-11T18:56:59.379027+00:00</t>
+          <t>2026-09-11T18:56:59.516665+00:00</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -13495,12 +13495,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>ALG-05</t>
+          <t>ALG-06</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O5</t>
         </is>
       </c>
       <c r="C247" t="inlineStr"/>
@@ -13508,27 +13508,27 @@
       <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Fold-safe scaling and preprocessing</t>
+          <t>Search based feature selection</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.txt</t>
+          <t>outputs/14_algorithms/ALG-06_search_based_feature_selection.txt</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>src/data_loader/splits.py; src/models/pipeline.py</t>
+          <t>src/feature_selection/ranking.py; src/feature_selection/sweep.py; src/optimization/base.py; src/optimization/multi_objective.py</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-05</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-06</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>2026-09-11T18:56:59.516665+00:00</t>
+          <t>2026-09-11T18:56:59.877724+00:00</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -13538,14 +13538,14 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>ALG-06</t>
+          <t>ALG-07</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -13558,27 +13558,27 @@
       <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Search based feature selection</t>
+          <t>Hyperparameter optimization</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-06_search_based_feature_selection.txt</t>
+          <t>outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>src/feature_selection/ranking.py; src/feature_selection/sweep.py; src/optimization/base.py; src/optimization/multi_objective.py</t>
+          <t>src/evaluation/tuned.py; src/optimization/base.py; src/optimization/bayesian.py</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-06</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-07</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>2026-09-11T18:56:59.877724+00:00</t>
+          <t>2026-09-11T18:57:00.038885+00:00</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -13588,19 +13588,19 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>ALG-07</t>
+          <t>ALG-08</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>O5</t>
+          <t>O3</t>
         </is>
       </c>
       <c r="C249" t="inlineStr"/>
@@ -13608,27 +13608,27 @@
       <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Hyperparameter optimization</t>
+          <t>SVM training and probability calibration</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt</t>
+          <t>outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.txt</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>src/evaluation/tuned.py; src/optimization/base.py; src/optimization/bayesian.py</t>
+          <t>src/models/calibration.py; src/models/estimators.py</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-07</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-08</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:00.038885+00:00</t>
+          <t>2026-09-11T18:57:01.375009+00:00</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -13638,14 +13638,14 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>ALG-08</t>
+          <t>ALG-09</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -13658,27 +13658,27 @@
       <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
-          <t>SVM training and probability calibration</t>
+          <t>Random Forest training</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.txt</t>
+          <t>outputs/14_algorithms/ALG-09_random_forest_training.txt</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>src/models/calibration.py; src/models/estimators.py</t>
+          <t>src/feature_selection/ranking.py; src/models/estimators.py; src/models/pipeline.py</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-08</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-09</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:01.375009+00:00</t>
+          <t>2026-09-11T18:57:01.523512+00:00</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -13688,14 +13688,14 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>ALG-09</t>
+          <t>ALG-10</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -13708,27 +13708,27 @@
       <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Random Forest training</t>
+          <t>Gradient Boosting training</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-09_random_forest_training.txt</t>
+          <t>outputs/14_algorithms/ALG-10_gradient_boosting_training.txt</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>src/feature_selection/ranking.py; src/models/estimators.py; src/models/pipeline.py</t>
+          <t>src/models/estimators.py; src/models/weighting.py</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-09</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-10</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:01.523512+00:00</t>
+          <t>2026-09-11T18:57:01.668016+00:00</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -13738,14 +13738,14 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>ALG-10</t>
+          <t>ALG-11</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -13758,27 +13758,27 @@
       <c r="E252" t="inlineStr"/>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Gradient Boosting training</t>
+          <t>Equal-weight soft voting</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-10_gradient_boosting_training.txt</t>
+          <t>outputs/14_algorithms/ALG-11_equal_weight_soft_voting.txt</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>src/models/estimators.py; src/models/weighting.py</t>
+          <t>src/ensemble/soft_voting.py; src/models/estimators.py</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-10</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-11</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:01.668016+00:00</t>
+          <t>2026-09-11T18:57:01.826498+00:00</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -13795,12 +13795,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>ALG-11</t>
+          <t>ALG-12</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>O3</t>
+          <t>O3, O5</t>
         </is>
       </c>
       <c r="C253" t="inlineStr"/>
@@ -13808,27 +13808,27 @@
       <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Equal-weight soft voting</t>
+          <t>Optimized-weight soft voting</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-11_equal_weight_soft_voting.txt</t>
+          <t>outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>src/ensemble/soft_voting.py; src/models/estimators.py</t>
+          <t>src/ensemble/soft_voting.py</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-11</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-12</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:01.826498+00:00</t>
+          <t>2026-09-11T18:57:01.961488+00:00</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -13838,19 +13838,19 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>ALG-12</t>
+          <t>ALG-13</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>O3, O5</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C254" t="inlineStr"/>
@@ -13858,27 +13858,27 @@
       <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Optimized-weight soft voting</t>
+          <t>Binary evaluation workflow</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt</t>
+          <t>outputs/14_algorithms/ALG-13_binary_evaluation_workflow.txt</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>src/ensemble/soft_voting.py</t>
+          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/evaluation/tuned.py</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-12</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-13</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:01.961488+00:00</t>
+          <t>2026-09-11T18:57:02.134574+00:00</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -13888,19 +13888,19 @@
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>ALG-13</t>
+          <t>ALG-14</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O6</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
@@ -13908,27 +13908,27 @@
       <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Binary evaluation workflow</t>
+          <t>Multiclass evaluation workflow</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-13_binary_evaluation_workflow.txt</t>
+          <t>outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.txt</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/evaluation/tuned.py</t>
+          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/reporting/multiclass_report.py</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-13</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-14</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:02.134574+00:00</t>
+          <t>2026-09-11T18:57:02.284549+00:00</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -13945,12 +13945,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>ALG-14</t>
+          <t>ALG-15</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>O6</t>
+          <t>O1, O3</t>
         </is>
       </c>
       <c r="C256" t="inlineStr"/>
@@ -13958,27 +13958,27 @@
       <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Multiclass evaluation workflow</t>
+          <t>CirCor subject-level aggregation</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.txt</t>
+          <t>outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.txt</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/reporting/multiclass_report.py</t>
+          <t>src/evaluation/aggregation.py</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-14</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-15</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:02.284549+00:00</t>
+          <t>2026-09-11T18:57:02.409665+00:00</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -13988,19 +13988,19 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>ALG-15</t>
+          <t>ALG-16</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>O1, O3</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C257" t="inlineStr"/>
@@ -14008,27 +14008,27 @@
       <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr">
         <is>
-          <t>CirCor subject-level aggregation</t>
+          <t>Cross-dataset external validation</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.txt</t>
+          <t>outputs/14_algorithms/ALG-16_cross_dataset_external_validation.txt</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>src/evaluation/aggregation.py</t>
+          <t>scripts/13_finalize_binary_model.py; src/evaluation/transfer.py; src/models/registry.py</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-15</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-16</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:02.409665+00:00</t>
+          <t>2026-09-11T18:57:02.542796+00:00</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -14038,19 +14038,19 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>ALG-16</t>
+          <t>ALG-17</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O4</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
@@ -14058,27 +14058,27 @@
       <c r="E258" t="inlineStr"/>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Cross-dataset external validation</t>
+          <t>Noise and duration robustness analysis</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-16_cross_dataset_external_validation.txt</t>
+          <t>outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.txt</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>scripts/13_finalize_binary_model.py; src/evaluation/transfer.py; src/models/registry.py</t>
+          <t>scripts/23_noise_robustness.py; scripts/24_duration_robustness.py; src/evaluation/duration.py; src/evaluation/robustness.py</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-16</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-17</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:02.542796+00:00</t>
+          <t>2026-09-11T18:57:02.695012+00:00</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>ALG-17</t>
+          <t>ALG-18</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O1, O4</t>
         </is>
       </c>
       <c r="C259" t="inlineStr"/>
@@ -14108,27 +14108,27 @@
       <c r="E259" t="inlineStr"/>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Noise and duration robustness analysis</t>
+          <t>Failure case analysis</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.txt</t>
+          <t>outputs/14_algorithms/ALG-18_failure_case_analysis.txt</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>scripts/23_noise_robustness.py; scripts/24_duration_robustness.py; src/evaluation/duration.py; src/evaluation/robustness.py</t>
+          <t>src/evaluation/failure_analysis.py; src/reporting/failure_report.py</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-17</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-18</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:02.695012+00:00</t>
+          <t>2026-09-11T18:57:02.844172+00:00</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -14138,19 +14138,19 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ALG-18</t>
+          <t>ALG-19</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>O1, O4</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C260" t="inlineStr"/>
@@ -14158,27 +14158,27 @@
       <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Failure case analysis</t>
+          <t>Sample-level report generation</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-18_failure_case_analysis.txt</t>
+          <t>outputs/14_algorithms/ALG-19_sample_level_report_generation.txt</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>src/evaluation/failure_analysis.py; src/reporting/failure_report.py</t>
+          <t>src/feature_extraction/extractor.py; src/inference/predictor.py; src/preprocessing/pipeline.py; src/reporting/sample_report.py</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-18</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-19</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:02.844172+00:00</t>
+          <t>2026-09-11T18:57:03.034105+00:00</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -14188,19 +14188,19 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>ALG-19</t>
+          <t>ALG-20</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O1-O6</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
@@ -14208,27 +14208,27 @@
       <c r="E261" t="inlineStr"/>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Sample-level report generation</t>
+          <t>Objective achievement evidence generation</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-19_sample_level_report_generation.txt</t>
+          <t>outputs/14_algorithms/ALG-20_objective_achievement_evidence_generation.txt</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>src/feature_extraction/extractor.py; src/inference/predictor.py; src/preprocessing/pipeline.py; src/reporting/sample_report.py</t>
+          <t>src/reporting/conclusion_tables.py; src/reporting/objectives.py; src/utils/evidence.py</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-19</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-20</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:03.034105+00:00</t>
+          <t>2026-09-11T18:57:03.163854+00:00</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -14238,19 +14238,19 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>ALG-20</t>
+          <t>MODEL-DEPLOY</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Deployment</t>
         </is>
       </c>
       <c r="C262" t="inlineStr"/>
@@ -14258,49 +14258,49 @@
       <c r="E262" t="inlineStr"/>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Objective achievement evidence generation</t>
+          <t>Deployed model per task: selection rule, ranking and hyperparameter source</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-20_objective_achievement_evidence_generation.txt</t>
+          <t>outputs/04_models/deployed_task_models.json</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>src/reporting/conclusion_tables.py; src/reporting/objectives.py; src/utils/evidence.py</t>
+          <t>outputs/07_multiclass_results/EXP-B2/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C1-three_class/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C2/aggregate_metrics.csv</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-20</t>
+          <t>python scripts/46_finalize_task_models.py</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:03.163854+00:00</t>
+          <t>2026-09-12T09:55:57.934243+00:00</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>source not on disk: outputs/07_multiclass_results/EXP-B2/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C1-three_class/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C2/aggregate_metrics.csv</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>THESIS-Ch1_Introduction</t>
+          <t>REPRO-01</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Reproducibility</t>
         </is>
       </c>
       <c r="C263" t="inlineStr"/>
@@ -14308,27 +14308,27 @@
       <c r="E263" t="inlineStr"/>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Ch1_Introduction: 9 diagram</t>
+          <t>T122.4 seed-discipline check: a re-run of EXP-B1-defaults against its committed aggregate metrics</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch1_Introduction/chapter_index.csv</t>
+          <t>outputs/00_evidence_index/reproducibility_check.json</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.svg; outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.png; outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.meta.json; outputs/13_figures_diagrams/F03_three_dataset_experimental_track_diagram.svg; outputs/13_figures_diagrams/F03_three_dataset_experimental_track_diagram.png; outputs/13_figures_diagrams/F03_three_dataset_experimental_track_diagram.meta.json; outputs/13_figures_diagrams/F19_novelty_contribution_diagram.svg; outputs/13_figures_diagrams/F19_novelty_contribution_diagram.png; outputs/13_figures_diagrams/F19_novelty_contribution_diagram.meta.json</t>
+          <t>outputs/07_multiclass_results/EXP-B1-defaults/aggregate_metrics.csv</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/11_run_experiment.py --exp EXP-B1 --variant defaults --out-dir &lt;scratch&gt; --no-resume</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.477098+00:00</t>
+          <t>2026-09-12T11:12:19.686335+00:00</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -14338,19 +14338,19 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>file and 9 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>THESIS-Ch2_Literature</t>
+          <t>SS-01</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C264" t="inlineStr"/>
@@ -14358,27 +14358,27 @@
       <c r="E264" t="inlineStr"/>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Ch2_Literature: 6 literature</t>
+          <t>Dashboard screenshot 1: Home and project overview</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch2_Literature/chapter_index.csv</t>
+          <t>outputs/15_dashboard_screenshots/SS-01_home.png</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>outputs/16_literature_review/LIT-01_literature_review_and_state_of_the_art.csv; outputs/16_literature_review/LIT-01_literature_review_and_state_of_the_art.docx; outputs/16_literature_review/LIT-01_literature_review_and_state_of_the_art.meta.json; outputs/16_literature_review/LIT-02_physionet_2016_published_comparison.csv; outputs/16_literature_review/LIT-02_physionet_2016_published_comparison.docx; outputs/16_literature_review/LIT-02_physionet_2016_published_comparison.meta.json</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.492781+00:00</t>
+          <t>2026-09-12T12:39:41.608380+00:00</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -14388,19 +14388,19 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>file and 6 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>THESIS-Ch3_Methodology</t>
+          <t>SS-02</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C265" t="inlineStr"/>
@@ -14408,27 +14408,27 @@
       <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Ch3_Methodology: 24 algorithm, 24 diagram, 3 equations, 30 graph, 21 table</t>
+          <t>Dashboard screenshot 2: Dataset inventory and class distribution</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch3_Methodology/chapter_index.csv</t>
+          <t>outputs/15_dashboard_screenshots/SS-02_dataset.png</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/T01_dataset_inventory.csv; outputs/01_dataset_audit/T01_dataset_inventory.docx; outputs/01_dataset_audit/T01_dataset_inventory.meta.json; outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.csv; outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.docx; outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.meta.json; outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.csv; outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.docx; outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.meta.json; outputs/02_preprocessing/T04_preprocessing_configuration.csv; outputs/02_preprocessing/T04_preprocessing_configuration.docx; outputs/02_preprocessing/T04_preprocessing_configuration.meta.json; outputs/03_features/T05_feature_inventory_and_counts.csv; outputs/03_features/T05_feature_inventory_and_counts.docx; outputs/03_features/T05_feature_inventory_and_counts.meta.json; outputs/04_models/T06_model_hyperparameter_configuration.csv; outputs/04_models/T06_model_hyperparameter_configuration.docx; outputs/04_models/T06_model_hyperparameter_configuration.meta.json; outputs/05_search_optimization/T07_search_space_and_best_parameters.csv; outputs/05_search_optimization/T07_search_space_and_best_parameters.docx; outputs/05_search_optimization/T07_search_space_and_best_parameters.meta.json; outputs/13_figures_diagrams/G01_dataset_recording_counts.png; outputs/13_figures_diagrams/G01_dataset_recording_counts.csv; outputs/13_figures_diagrams/G01_dataset_recording_counts.meta.json; outputs/13_figures_diagrams/G02_class_distribution.png; outputs/13_figures_diagrams/G02_class_distribution.csv; outputs/13_figures_diagrams/G02_class_distribution.meta.json; outputs/13_figures_diagrams/G03_class_distribution_shares.png; outputs/13_figures_diagrams/G03_class_distribution_shares.csv; outputs/13_figures_diagrams/G03_class_distribution_shares.meta.json; outputs/13_figures_diagrams/G04_recording_duration_histogram.png; outputs/13_figures_diagrams/G04_recording_duration_histogram.csv; outputs/13_figures_diagrams/G04_recording_duration_histogram.meta.json; outputs/13_figures_diagrams/G05_before_and_after_filtering.png; outputs/13_figures_diagrams/G05_before_and_after_filtering.csv; outputs/13_figures_diagrams/G05_before_and_after_filtering.meta.json; outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.png; outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.csv; outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.meta.json; outputs/13_figures_diagrams/G07_mfcc_heatmap.png; outputs/13_figures_diagrams/G07_mfcc_heatmap.csv; outputs/13_figures_diagrams/G07_mfcc_heatmap.meta.json; outputs/13_figures_diagrams/G08_chroma_heatmap.png; outputs/13_figures_diagrams/G08_chroma_heatmap.csv; outputs/13_figures_diagrams/G08_chroma_heatmap.meta.json; outputs/13_figures_diagrams/G09_wavelet_decomposition.png; outputs/13_figures_diagrams/G09_wavelet_decomposition.csv; outputs/13_figures_diagrams/G09_wavelet_decomposition.meta.json; outputs/13_figures_diagrams/G10_feature_family_counts.png; outputs/13_figures_diagrams/G10_feature_family_counts.csv; outputs/13_figures_diagrams/G10_feature_family_counts.meta.json; outputs/13_figures_diagrams/F02_end_to_end_pcg_classification_workflow.svg; outputs/13_figures_diagrams/F02_end_to_end_pcg_classification_workflow.png; outputs/13_figures_diagrams/F02_end_to_end_pcg_classification_workflow.meta.json; outputs/13_figures_diagrams/F04_dataset_harmonization_and_metadata_workflow.svg; outputs/13_figures_diagrams/F04_dataset_harmonization_and_metadata_workflow.png; outputs/13_figures_diagrams/F04_dataset_harmonization_and_metadata_workflow.meta.json; outputs/13_figures_diagrams/F05_subject_wise_data_splitting.svg; outputs/13_figures_diagrams/F05_subject_wise_data_splitting.png; outputs/13_figures_diagrams/F05_subject_wise_data_splitting.meta.json; outputs/13_figures_diagrams/F06_signal_preprocessing_architecture.svg; outputs/13_figures_diagrams/F06_signal_preprocessing_architecture.png; outputs/13_figures_diagrams/F06_signal_preprocessing_architecture.meta.json; outputs/13_figures_diagrams/F07_138_feature_extraction_architecture.svg; outputs/13_figures_diagrams/F07_138_feature_extraction_architecture.png; outputs/13_figures_diagrams/F07_138_feature_extraction_architecture.meta.json; outputs/13_figures_diagrams/F08_feature_family_fusion.svg; outputs/13_figures_diagrams/F08_feature_family_fusion.png; outputs/13_figures_diagrams/F08_feature_family_fusion.meta.json; outputs/13_figures_diagrams/F09_search_based_feature_selection_workflow.svg; outputs/13_figures_diagrams/F09_search_based_feature_selection_workflow.png; outputs/13_figures_diagrams/F09_search_based_feature_selection_workflow.meta.json; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.svg; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.png; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.meta.json; outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.docx; outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.txt; outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.docx; outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.txt; outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.docx; outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.txt; outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.docx; outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt; outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.docx; outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.txt; outputs/14_algorithms/ALG-06_search_based_feature_selection.docx; outputs/14_algorithms/ALG-06_search_based_feature_selection.txt; outputs/14_algorithms/ALG-07_hyperparameter_optimization.docx; outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt; outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.docx; outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.txt; outputs/14_algorithms/ALG-09_random_forest_training.docx; outputs/14_algorithms/ALG-09_random_forest_training.txt; outputs/14_algorithms/ALG-10_gradient_boosting_training.docx; outputs/14_algorithms/ALG-10_gradient_boosting_training.txt; outputs/14_algorithms/ALG-11_equal_weight_soft_voting.docx; outputs/14_algorithms/ALG-11_equal_weight_soft_voting.txt; outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.docx; outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt; outputs/14_algorithms/equations_reference.docx; outputs/14_algorithms/equations_reference.tex; outputs/14_algorithms/equations_reference.csv</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.549509+00:00</t>
+          <t>2026-09-12T12:39:41.687661+00:00</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -14438,19 +14438,19 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>file and 102 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>THESIS-Ch4_Implementation</t>
+          <t>SS-03</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C266" t="inlineStr"/>
@@ -14458,27 +14458,27 @@
       <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Ch4_Implementation: 14 algorithm, 1 appendix, 21 diagram</t>
+          <t>Dashboard screenshot 3: Signal upload and waveform</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch4_Implementation/chapter_index.csv</t>
+          <t>outputs/15_dashboard_screenshots/SS-03_predict_binary.png</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/F11_binary_classification_pipeline.svg; outputs/13_figures_diagrams/F11_binary_classification_pipeline.png; outputs/13_figures_diagrams/F11_binary_classification_pipeline.meta.json; outputs/13_figures_diagrams/F12_pascal_multiclass_pipeline.svg; outputs/13_figures_diagrams/F12_pascal_multiclass_pipeline.png; outputs/13_figures_diagrams/F12_pascal_multiclass_pipeline.meta.json; outputs/13_figures_diagrams/F13_circor_recording_to_subject_aggregation.svg; outputs/13_figures_diagrams/F13_circor_recording_to_subject_aggregation.png; outputs/13_figures_diagrams/F13_circor_recording_to_subject_aggregation.meta.json; outputs/13_figures_diagrams/F14_cross_dataset_external_validation_workflow.svg; outputs/13_figures_diagrams/F14_cross_dataset_external_validation_workflow.png; outputs/13_figures_diagrams/F14_cross_dataset_external_validation_workflow.meta.json; outputs/13_figures_diagrams/F15_noise_and_duration_robustness_framework.svg; outputs/13_figures_diagrams/F15_noise_and_duration_robustness_framework.png; outputs/13_figures_diagrams/F15_noise_and_duration_robustness_framework.meta.json; outputs/13_figures_diagrams/F16_dashboard_system_architecture.svg; outputs/13_figures_diagrams/F16_dashboard_system_architecture.png; outputs/13_figures_diagrams/F16_dashboard_system_architecture.meta.json; outputs/13_figures_diagrams/F17_prediction_and_report_generation_flow.svg; outputs/13_figures_diagrams/F17_prediction_and_report_generation_flow.png; outputs/13_figures_diagrams/F17_prediction_and_report_generation_flow.meta.json; outputs/14_algorithms/ALG-13_binary_evaluation_workflow.docx; outputs/14_algorithms/ALG-13_binary_evaluation_workflow.txt; outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.docx; outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.txt; outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.docx; outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.txt; outputs/14_algorithms/ALG-16_cross_dataset_external_validation.docx; outputs/14_algorithms/ALG-16_cross_dataset_external_validation.txt; outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.docx; outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.txt; outputs/14_algorithms/ALG-18_failure_case_analysis.docx; outputs/14_algorithms/ALG-18_failure_case_analysis.txt; outputs/14_algorithms/ALG-19_sample_level_report_generation.docx; outputs/14_algorithms/ALG-19_sample_level_report_generation.txt; outputs/00_evidence_index/run_manifest.json; outputs/00_evidence_index/evidence_index.csv</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.574232+00:00</t>
+          <t>2026-09-12T12:39:41.703676+00:00</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -14488,19 +14488,19 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>file and 37 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>THESIS-Ch5_Results</t>
+          <t>SS-04</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C267" t="inlineStr"/>
@@ -14508,27 +14508,27 @@
       <c r="E267" t="inlineStr"/>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Ch5_Results: 75 graph, 63 table</t>
+          <t>Dashboard screenshot 4: Preprocessing before/after</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch5_Results/chapter_index.csv</t>
+          <t>outputs/15_dashboard_screenshots/SS-04_preprocessing.png</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>outputs/06_binary_results/T08_physionet_individual_model_comparison.csv; outputs/06_binary_results/T08_physionet_individual_model_comparison.docx; outputs/06_binary_results/T08_physionet_individual_model_comparison.meta.json; outputs/06_binary_results/T09_equal_weight_versus_optimized_ensemble.csv; outputs/06_binary_results/T09_equal_weight_versus_optimized_ensemble.docx; outputs/06_binary_results/T09_equal_weight_versus_optimized_ensemble.meta.json; outputs/06_binary_results/T10_physionet_fold_wise_results.csv; outputs/06_binary_results/T10_physionet_fold_wise_results.docx; outputs/06_binary_results/T10_physionet_fold_wise_results.meta.json; outputs/07_multiclass_results/T11_pascal_a_multiclass_results.csv; outputs/07_multiclass_results/T11_pascal_a_multiclass_results.docx; outputs/07_multiclass_results/T11_pascal_a_multiclass_results.meta.json; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.csv; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.docx; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.meta.json; outputs/08_circor_external_validation/T13_circor_murmur_classification_results.csv; outputs/08_circor_external_validation/T13_circor_murmur_classification_results.docx; outputs/08_circor_external_validation/T13_circor_murmur_classification_results.meta.json; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.csv; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.docx; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.meta.json; outputs/08_circor_external_validation/T15_recording_level_versus_subject_level_results.csv; outputs/08_circor_external_validation/T15_recording_level_versus_subject_level_results.docx; outputs/08_circor_external_validation/T15_recording_level_versus_subject_level_results.meta.json; outputs/08_circor_external_validation/T16_cross_dataset_generalization.csv; outputs/08_circor_external_validation/T16_cross_dataset_generalization.docx; outputs/08_circor_external_validation/T16_cross_dataset_generalization.meta.json; outputs/09_ablation/T17_feature_family_ablation.csv; outputs/09_ablation/T17_feature_family_ablation.docx; outputs/09_ablation/T17_feature_family_ablation.meta.json; outputs/09_ablation/T18_all_features_versus_selected_features.csv; outputs/09_ablation/T18_all_features_versus_selected_features.docx; outputs/09_ablation/T18_all_features_versus_selected_features.meta.json; outputs/09_ablation/T19_search_and_optimization_ablation.csv; outputs/09_ablation/T19_search_and_optimization_ablation.docx; outputs/09_ablation/T19_search_and_optimization_ablation.meta.json; outputs/09_robustness_analysis/T20_noise_robustness.csv; outputs/09_robustness_analysis/T20_noise_robustness.docx; outputs/09_robustness_analysis/T20_noise_robustness.meta.json; outputs/09_robustness_analysis/T21_duration_robustness.csv; outputs/09_robustness_analysis/T21_duration_robustness.docx; outputs/09_robustness_analysis/T21_duration_robustness.meta.json; outputs/08_circor_external_validation/T22_auscultation_location_analysis.csv; outputs/08_circor_external_validation/T22_auscultation_location_analysis.docx; outputs/08_circor_external_validation/T22_auscultation_location_analysis.meta.json; outputs/10_robustness/T23_calibration_and_confidence_summary.csv; outputs/10_robustness/T23_calibration_and_confidence_summary.docx; outputs/10_robustness/T23_calibration_and_confidence_summary.meta.json; outputs/11_complexity/T24_complexity_analysis.csv; outputs/11_complexity/T24_complexity_analysis.docx; outputs/11_complexity/T24_complexity_analysis.meta.json; outputs/11_complexity/T25_training_and_inference_time.csv; outputs/11_complexity/T25_training_and_inference_time.docx; outputs/11_complexity/T25_training_and_inference_time.meta.json; outputs/11_complexity/T26_model_size_and_memory.csv; outputs/11_complexity/T26_model_size_and_memory.docx; outputs/11_complexity/T26_model_size_and_memory.meta.json; outputs/10_robustness/T27_false_positive_and_false_negative_analysis.csv; outputs/10_robustness/T27_false_positive_and_false_negative_analysis.docx; outputs/10_robustness/T27_false_positive_and_false_negative_analysis.meta.json; outputs/12_statistics/T28_statistical_significance_comparison.csv; outputs/12_statistics/T28_statistical_significance_comparison.docx; outputs/12_statistics/T28_statistical_significance_comparison.meta.json; outputs/13_figures_diagrams/G11_individual_model_comparison.png; outputs/13_figures_diagrams/G11_individual_model_comparison.csv; outputs/13_figures_diagrams/G11_individual_model_comparison.meta.json; outputs/13_figures_diagrams/G12_binary_roc_curve.png; outputs/13_figures_diagrams/G12_binary_roc_curve.csv; outputs/13_figures_diagrams/G12_binary_roc_curve.meta.json; outputs/13_figures_diagrams/G13_binary_precision_recall_curve.png; outputs/13_figures_diagrams/G13_binary_precision_recall_curve.csv; outputs/13_figures_diagrams/G13_binary_precision_recall_curve.meta.json; outputs/13_figures_diagrams/G14_binary_confusion_matrix.png; outputs/13_figures_diagrams/G14_binary_confusion_matrix.csv; outputs/13_figures_diagrams/G14_binary_confusion_matrix.meta.json; outputs/13_figures_diagrams/G15_pascal_a_confusion_matrix.png; outputs/13_figures_diagrams/G15_pascal_a_confusion_matrix.csv; outputs/13_figures_diagrams/G15_pascal_a_confusion_matrix.meta.json; outputs/13_figures_diagrams/G16_pascal_b_confusion_matrix.png; outputs/13_figures_diagrams/G16_pascal_b_confusion_matrix.csv; outputs/13_figures_diagrams/G16_pascal_b_confusion_matrix.meta.json; outputs/13_figures_diagrams/G17_multiclass_one_vs_rest_roc.png; outputs/13_figures_diagrams/G17_multiclass_one_vs_rest_roc.csv; outputs/13_figures_diagrams/G17_multiclass_one_vs_rest_roc.meta.json; outputs/13_figures_diagrams/G18_feature_importance_plot.png; outputs/13_figures_diagrams/G18_feature_importance_plot.csv; outputs/13_figures_diagrams/G18_feature_importance_plot.meta.json; outputs/13_figures_diagrams/G19_top_20_features_chart.png; outputs/13_figures_diagrams/G19_top_20_features_chart.csv; outputs/13_figures_diagrams/G19_top_20_features_chart.meta.json; outputs/13_figures_diagrams/G20_search_convergence_plot.png; outputs/13_figures_diagrams/G20_search_convergence_plot.csv; outputs/13_figures_diagrams/G20_search_convergence_plot.meta.json; outputs/13_figures_diagrams/G21_all_features_versus_selected_features.png; outputs/13_figures_diagrams/G21_all_features_versus_selected_features.csv; outputs/13_figures_diagrams/G21_all_features_versus_selected_features.meta.json; outputs/13_figures_diagrams/G22_f1_and_accuracy_versus_feature_count.png; outputs/13_figures_diagrams/G22_f1_and_accuracy_versus_feature_count.csv; outputs/13_figures_diagrams/G22_f1_and_accuracy_versus_feature_count.meta.json; outputs/13_figures_diagrams/G23_ensemble_weight_comparison.png; outputs/13_figures_diagrams/G23_ensemble_weight_comparison.csv; outputs/13_figures_diagrams/G23_ensemble_weight_comparison.meta.json; outputs/13_figures_diagrams/G24_baseline_versus_optimized.png; outputs/13_figures_diagrams/G24_baseline_versus_optimized.csv; outputs/13_figures_diagrams/G24_baseline_versus_optimized.meta.json; outputs/13_figures_diagrams/G25_inference_time_versus_performance.png; outputs/13_figures_diagrams/G25_inference_time_versus_performance.csv; outputs/13_figures_diagrams/G25_inference_time_versus_performance.meta.json; outputs/13_figures_diagrams/G26_training_time_comparison.png; outputs/13_figures_diagrams/G26_training_time_comparison.csv; outputs/13_figures_diagrams/G26_training_time_comparison.meta.json; outputs/13_figures_diagrams/G27_model_size_comparison.png; outputs/13_figures_diagrams/G27_model_size_comparison.csv; outputs/13_figures_diagrams/G27_model_size_comparison.meta.json; outputs/13_figures_diagrams/G28_dataset_wise_generalization.png; outputs/13_figures_diagrams/G28_dataset_wise_generalization.csv; outputs/13_figures_diagrams/G28_dataset_wise_generalization.meta.json; outputs/13_figures_diagrams/G29_cross_dataset_performance_drop.png; outputs/13_figures_diagrams/G29_cross_dataset_performance_drop.csv; outputs/13_figures_diagrams/G29_cross_dataset_performance_drop.meta.json; outputs/13_figures_diagrams/G30_noise_level_robustness.png; outputs/13_figures_diagrams/G30_noise_level_robustness.csv; outputs/13_figures_diagrams/G30_noise_level_robustness.meta.json; outputs/13_figures_diagrams/G31_duration_wise_performance.png; outputs/13_figures_diagrams/G31_duration_wise_performance.csv; outputs/13_figures_diagrams/G31_duration_wise_performance.meta.json; outputs/13_figures_diagrams/G32_location_performance.png; outputs/13_figures_diagrams/G32_location_performance.csv; outputs/13_figures_diagrams/G32_location_performance.meta.json; outputs/13_figures_diagrams/G33_confidence_histogram.png; outputs/13_figures_diagrams/G33_confidence_histogram.csv; outputs/13_figures_diagrams/G33_confidence_histogram.meta.json; outputs/13_figures_diagrams/G34_calibration_curve.png; outputs/13_figures_diagrams/G34_calibration_curve.csv; outputs/13_figures_diagrams/G34_calibration_curve.meta.json; outputs/13_figures_diagrams/G35_false_positive_and_false_negative_distribution.png; outputs/13_figures_diagrams/G35_false_positive_and_false_negative_distribution.csv; outputs/13_figures_diagrams/G35_false_positive_and_false_negative_distribution.meta.json</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.635621+00:00</t>
+          <t>2026-09-12T12:39:41.736716+00:00</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -14538,19 +14538,19 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>file and 138 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>THESIS-Ch6_Conclusion</t>
+          <t>SS-05</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C268" t="inlineStr"/>
@@ -14558,27 +14558,27 @@
       <c r="E268" t="inlineStr"/>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Ch6_Conclusion: 2 algorithm, 6 diagram, 6 table</t>
+          <t>Dashboard screenshot 5: Feature extraction summary</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch6_Conclusion/chapter_index.csv</t>
+          <t>outputs/15_dashboard_screenshots/SS-05_features.png</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>outputs/00_evidence_index/T29_objective_to_evidence_mapping.csv; outputs/00_evidence_index/T29_objective_to_evidence_mapping.docx; outputs/00_evidence_index/T29_objective_to_evidence_mapping.meta.json; outputs/00_evidence_index/T30_final_conclusion_matrix.csv; outputs/00_evidence_index/T30_final_conclusion_matrix.docx; outputs/00_evidence_index/T30_final_conclusion_matrix.meta.json; outputs/13_figures_diagrams/F18_objective_to_module_traceability.svg; outputs/13_figures_diagrams/F18_objective_to_module_traceability.png; outputs/13_figures_diagrams/F18_objective_to_module_traceability.meta.json; outputs/13_figures_diagrams/F20_final_research_contribution_summary.svg; outputs/13_figures_diagrams/F20_final_research_contribution_summary.png; outputs/13_figures_diagrams/F20_final_research_contribution_summary.meta.json; outputs/14_algorithms/ALG-20_objective_achievement_evidence_generation.docx; outputs/14_algorithms/ALG-20_objective_achievement_evidence_generation.txt</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.658943+00:00</t>
+          <t>2026-09-12T12:39:41.751496+00:00</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -14588,43 +14588,47 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>file and 14 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>THESIS-REPRODUCIBILITY</t>
-        </is>
-      </c>
-      <c r="B269" t="inlineStr"/>
+          <t>SS-06</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
       <c r="C269" t="inlineStr"/>
       <c r="D269" t="inlineStr"/>
       <c r="E269" t="inlineStr"/>
       <c r="F269" t="inlineStr">
         <is>
-          <t>reproducibility appendix: environment, seeds, packages, stage timing, commands</t>
+          <t>Dashboard screenshot 6: Model comparison dashboard</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>outputs/THESIS_ASSETS/Ch4_Implementation/reproducibility_appendix.docx</t>
+          <t>outputs/15_dashboard_screenshots/SS-06_models.png</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>outputs/00_evidence_index/run_manifest.json</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>python scripts/44_thesis_assets.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>2026-09-11T18:57:10.675668+00:00</t>
+          <t>2026-09-12T12:39:41.780007+00:00</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -14634,19 +14638,19 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>MODEL-DEPLOY</t>
+          <t>SS-07</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C270" t="inlineStr"/>
@@ -14654,49 +14658,49 @@
       <c r="E270" t="inlineStr"/>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Deployed model per task: selection rule, ranking and hyperparameter source</t>
+          <t>Dashboard screenshot 7: Search optimization dashboard</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>outputs/04_models/deployed_task_models.json</t>
+          <t>outputs/15_dashboard_screenshots/SS-07_optimization.png</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>outputs/07_multiclass_results/EXP-B2/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C1-three_class/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C2/aggregate_metrics.csv</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>python scripts/46_finalize_task_models.py</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>2026-09-12T09:55:57.934243+00:00</t>
+          <t>2026-09-12T12:39:41.804007+00:00</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>source not on disk: outputs/07_multiclass_results/EXP-B2/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C1-three_class/aggregate_metrics.csv,outputs/08_circor_external_validation/EXP-C2/aggregate_metrics.csv</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>REPRO-01</t>
+          <t>SS-08</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Reproducibility</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C271" t="inlineStr"/>
@@ -14704,27 +14708,27 @@
       <c r="E271" t="inlineStr"/>
       <c r="F271" t="inlineStr">
         <is>
-          <t>T122.4 seed-discipline check: a re-run of EXP-B1-defaults against its committed aggregate metrics</t>
+          <t>Dashboard screenshot 8: Binary prediction output</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>outputs/00_evidence_index/reproducibility_check.json</t>
+          <t>outputs/15_dashboard_screenshots/SS-08_predict_binary.png</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>outputs/07_multiclass_results/EXP-B1-defaults/aggregate_metrics.csv</t>
+          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>python scripts/11_run_experiment.py --exp EXP-B1 --variant defaults --out-dir &lt;scratch&gt; --no-resume</t>
+          <t>python scripts/47_dashboard_screenshots.py</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>2026-09-12T11:12:19.686335+00:00</t>
+          <t>2026-09-12T12:39:41.829957+00:00</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -14734,14 +14738,14 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file on disk; source is descriptive, not a path</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>SS-01</t>
+          <t>SS-09</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -14754,12 +14758,12 @@
       <c r="E272" t="inlineStr"/>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 1: Home and project overview</t>
+          <t>Dashboard screenshot 9: Multiclass prediction output</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-01_home.png</t>
+          <t>outputs/15_dashboard_screenshots/SS-09_predict_multiclass.png</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -14774,7 +14778,7 @@
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.608380+00:00</t>
+          <t>2026-09-12T12:39:41.852384+00:00</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -14791,7 +14795,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>SS-02</t>
+          <t>SS-10</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -14804,12 +14808,12 @@
       <c r="E273" t="inlineStr"/>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 2: Dataset inventory and class distribution</t>
+          <t>Dashboard screenshot 10: CirCor murmur/outcome output</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-02_dataset.png</t>
+          <t>outputs/15_dashboard_screenshots/SS-10_predict_murmur.png</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
@@ -14824,7 +14828,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.687661+00:00</t>
+          <t>2026-09-12T12:39:41.880585+00:00</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -14841,7 +14845,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>SS-03</t>
+          <t>SS-11</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -14854,12 +14858,12 @@
       <c r="E274" t="inlineStr"/>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 3: Signal upload and waveform</t>
+          <t>Dashboard screenshot 11: Robustness analytics</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-03_predict_binary.png</t>
+          <t>outputs/15_dashboard_screenshots/SS-11_robustness.png</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -14874,7 +14878,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.703676+00:00</t>
+          <t>2026-09-12T12:39:41.904323+00:00</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -14891,7 +14895,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>SS-04</t>
+          <t>SS-12</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -14904,12 +14908,12 @@
       <c r="E275" t="inlineStr"/>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 4: Preprocessing before/after</t>
+          <t>Dashboard screenshot 12: Feature importance/explainability</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-04_preprocessing.png</t>
+          <t>outputs/15_dashboard_screenshots/SS-12_explainability.png</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -14924,7 +14928,7 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.736716+00:00</t>
+          <t>2026-09-12T12:39:41.923851+00:00</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -14941,7 +14945,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>SS-05</t>
+          <t>SS-13</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -14954,12 +14958,12 @@
       <c r="E276" t="inlineStr"/>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 5: Feature extraction summary</t>
+          <t>Dashboard screenshot 13: Exported report preview</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-05_features.png</t>
+          <t>outputs/15_dashboard_screenshots/SS-13_reports.png</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -14974,7 +14978,7 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.751496+00:00</t>
+          <t>2026-09-12T12:39:41.946596+00:00</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -14991,7 +14995,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>SS-06</t>
+          <t>SS-INDEX</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -15004,17 +15008,17 @@
       <c r="E277" t="inlineStr"/>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 6: Model comparison dashboard</t>
+          <t>Dashboard screenshot index with captions</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-06_models.png</t>
+          <t>outputs/15_dashboard_screenshots/screenshot_index.csv</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
+          <t>outputs/15_dashboard_screenshots/capture_plan.json</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -15024,7 +15028,7 @@
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.780007+00:00</t>
+          <t>2026-09-12T12:39:41.975706+00:00</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -15034,247 +15038,211 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>SS-07</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
+          <t>QA-SWEEP</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr"/>
       <c r="C278" t="inlineStr"/>
       <c r="D278" t="inlineStr"/>
       <c r="E278" t="inlineStr"/>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 7: Search optimization dashboard</t>
+          <t>final QA sweep across six areas (Phase 124)</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-07_optimization.png</t>
-        </is>
-      </c>
-      <c r="H278" t="inlineStr">
-        <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
-        </is>
-      </c>
+          <t>outputs/00_evidence_index/final_qa_report.md</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/49_final_qa_sweep.py</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.804007+00:00</t>
+          <t>2026-09-12T14:09:12.050185+00:00</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>no source_data recorded</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>SS-08</t>
-        </is>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
+          <t>QA-COMPLIANCE</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr"/>
       <c r="C279" t="inlineStr"/>
       <c r="D279" t="inlineStr"/>
       <c r="E279" t="inlineStr"/>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 8: Binary prediction output</t>
+          <t>compliance and claims review (Phase 125)</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-08_predict_binary.png</t>
-        </is>
-      </c>
-      <c r="H279" t="inlineStr">
-        <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
-        </is>
-      </c>
+          <t>outputs/00_evidence_index/compliance_review.md</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/50_compliance_review.py</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.829957+00:00</t>
+          <t>2026-09-12T14:10:21.244861+00:00</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>no source_data recorded</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>SS-09</t>
-        </is>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
+          <t>DOC-HANDOVER</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr"/>
       <c r="C280" t="inlineStr"/>
       <c r="D280" t="inlineStr"/>
       <c r="E280" t="inlineStr"/>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 9: Multiclass prediction output</t>
+          <t>handover summary: produced, not produced, next steps (T126.6)</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-09_predict_multiclass.png</t>
-        </is>
-      </c>
-      <c r="H280" t="inlineStr">
-        <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
-        </is>
-      </c>
+          <t>HANDOVER.md</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr"/>
       <c r="I280" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/51_package_delivery.py</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.852384+00:00</t>
+          <t>2026-09-12T15:32:49.621460+00:00</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>no source_data recorded</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>SS-10</t>
-        </is>
-      </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
+          <t>DOC-ARCH</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr"/>
       <c r="C281" t="inlineStr"/>
       <c r="D281" t="inlineStr"/>
       <c r="E281" t="inlineStr"/>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 10: CirCor murmur/outcome output</t>
+          <t>project structure and the role of each module (T123.2)</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-10_predict_murmur.png</t>
-        </is>
-      </c>
-      <c r="H281" t="inlineStr">
-        <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
-        </is>
-      </c>
+          <t>ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr"/>
       <c r="I281" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/48_project_docs.py</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.880585+00:00</t>
+          <t>2026-09-13T19:14:30.579200+00:00</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>no source_data recorded</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>SS-11</t>
-        </is>
-      </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
+          <t>DOC-CONFIG</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr"/>
       <c r="C282" t="inlineStr"/>
       <c r="D282" t="inlineStr"/>
       <c r="E282" t="inlineStr"/>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 11: Robustness analytics</t>
+          <t>every configuration option and its default (T123.3)</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-11_robustness.png</t>
+          <t>CONFIGURATION.md</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
+          <t>configs</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/48_project_docs.py</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.904323+00:00</t>
+          <t>2026-09-13T19:14:30.658601+00:00</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -15291,12 +15259,12 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>SS-12</t>
+          <t>F16</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
@@ -15304,27 +15272,27 @@
       <c r="E283" t="inlineStr"/>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 12: Feature importance/explainability</t>
+          <t>Dashboard system architecture</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-12_explainability.png</t>
+          <t>outputs/13_figures_diagrams/F16_dashboard_system_architecture.png</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
+          <t>src/reporting/diagrams/pipeline_figures.py</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/05_render_diagrams.py --only F16</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.923851+00:00</t>
+          <t>2026-09-14T06:57:31.724955+00:00</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -15334,19 +15302,19 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>SS-13</t>
+          <t>THESIS-Ch1_Introduction</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>O1-O6</t>
         </is>
       </c>
       <c r="C284" t="inlineStr"/>
@@ -15354,27 +15322,27 @@
       <c r="E284" t="inlineStr"/>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Dashboard screenshot 13: Exported report preview</t>
+          <t>Ch1_Introduction: 9 diagram</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/SS-13_reports.png</t>
+          <t>outputs/THESIS_ASSETS/Ch1_Introduction/chapter_index.csv</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>frontend/lib/generated (build-time codegen from outputs/)</t>
+          <t>outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.svg; outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.png; outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.meta.json; outputs/13_figures_diagrams/F03_three_dataset_experimental_track_diagram.svg; outputs/13_figures_diagrams/F03_three_dataset_experimental_track_diagram.png; outputs/13_figures_diagrams/F03_three_dataset_experimental_track_diagram.meta.json; outputs/13_figures_diagrams/F19_novelty_contribution_diagram.svg; outputs/13_figures_diagrams/F19_novelty_contribution_diagram.png; outputs/13_figures_diagrams/F19_novelty_contribution_diagram.meta.json</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.946596+00:00</t>
+          <t>2026-09-14T06:58:00.652545+00:00</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -15384,19 +15352,19 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>file and 9 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>SS-INDEX</t>
+          <t>THESIS-Ch2_Literature</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>O1-O6</t>
         </is>
       </c>
       <c r="C285" t="inlineStr"/>
@@ -15404,27 +15372,27 @@
       <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Dashboard screenshot index with captions</t>
+          <t>Ch2_Literature: 6 literature</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/screenshot_index.csv</t>
+          <t>outputs/THESIS_ASSETS/Ch2_Literature/chapter_index.csv</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>outputs/15_dashboard_screenshots/capture_plan.json</t>
+          <t>outputs/16_literature_review/LIT-01_literature_review_and_state_of_the_art.csv; outputs/16_literature_review/LIT-01_literature_review_and_state_of_the_art.docx; outputs/16_literature_review/LIT-01_literature_review_and_state_of_the_art.meta.json; outputs/16_literature_review/LIT-02_physionet_2016_published_comparison.csv; outputs/16_literature_review/LIT-02_physionet_2016_published_comparison.docx; outputs/16_literature_review/LIT-02_physionet_2016_published_comparison.meta.json</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>python scripts/47_dashboard_screenshots.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>2026-09-12T12:39:41.975706+00:00</t>
+          <t>2026-09-14T06:58:00.667352+00:00</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -15434,169 +15402,197 @@
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 6 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>QA-SWEEP</t>
-        </is>
-      </c>
-      <c r="B286" t="inlineStr"/>
+          <t>THESIS-Ch3_Methodology</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>O1-O6</t>
+        </is>
+      </c>
       <c r="C286" t="inlineStr"/>
       <c r="D286" t="inlineStr"/>
       <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr">
         <is>
-          <t>final QA sweep across six areas (Phase 124)</t>
+          <t>Ch3_Methodology: 24 algorithm, 24 diagram, 3 equations, 30 graph, 21 table</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>outputs/00_evidence_index/final_qa_report.md</t>
-        </is>
-      </c>
-      <c r="H286" t="inlineStr"/>
+          <t>outputs/THESIS_ASSETS/Ch3_Methodology/chapter_index.csv</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>outputs/01_dataset_audit/T01_dataset_inventory.csv; outputs/01_dataset_audit/T01_dataset_inventory.docx; outputs/01_dataset_audit/T01_dataset_inventory.meta.json; outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.csv; outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.docx; outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.meta.json; outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.csv; outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.docx; outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.meta.json; outputs/02_preprocessing/T04_preprocessing_configuration.csv; outputs/02_preprocessing/T04_preprocessing_configuration.docx; outputs/02_preprocessing/T04_preprocessing_configuration.meta.json; outputs/03_features/T05_feature_inventory_and_counts.csv; outputs/03_features/T05_feature_inventory_and_counts.docx; outputs/03_features/T05_feature_inventory_and_counts.meta.json; outputs/04_models/T06_model_hyperparameter_configuration.csv; outputs/04_models/T06_model_hyperparameter_configuration.docx; outputs/04_models/T06_model_hyperparameter_configuration.meta.json; outputs/05_search_optimization/T07_search_space_and_best_parameters.csv; outputs/05_search_optimization/T07_search_space_and_best_parameters.docx; outputs/05_search_optimization/T07_search_space_and_best_parameters.meta.json; outputs/13_figures_diagrams/G01_dataset_recording_counts.png; outputs/13_figures_diagrams/G01_dataset_recording_counts.csv; outputs/13_figures_diagrams/G01_dataset_recording_counts.meta.json; outputs/13_figures_diagrams/G02_class_distribution.png; outputs/13_figures_diagrams/G02_class_distribution.csv; outputs/13_figures_diagrams/G02_class_distribution.meta.json; outputs/13_figures_diagrams/G03_class_distribution_shares.png; outputs/13_figures_diagrams/G03_class_distribution_shares.csv; outputs/13_figures_diagrams/G03_class_distribution_shares.meta.json; outputs/13_figures_diagrams/G04_recording_duration_histogram.png; outputs/13_figures_diagrams/G04_recording_duration_histogram.csv; outputs/13_figures_diagrams/G04_recording_duration_histogram.meta.json; outputs/13_figures_diagrams/G05_before_and_after_filtering.png; outputs/13_figures_diagrams/G05_before_and_after_filtering.csv; outputs/13_figures_diagrams/G05_before_and_after_filtering.meta.json; outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.png; outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.csv; outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.meta.json; outputs/13_figures_diagrams/G07_mfcc_heatmap.png; outputs/13_figures_diagrams/G07_mfcc_heatmap.csv; outputs/13_figures_diagrams/G07_mfcc_heatmap.meta.json; outputs/13_figures_diagrams/G08_chroma_heatmap.png; outputs/13_figures_diagrams/G08_chroma_heatmap.csv; outputs/13_figures_diagrams/G08_chroma_heatmap.meta.json; outputs/13_figures_diagrams/G09_wavelet_decomposition.png; outputs/13_figures_diagrams/G09_wavelet_decomposition.csv; outputs/13_figures_diagrams/G09_wavelet_decomposition.meta.json; outputs/13_figures_diagrams/G10_feature_family_counts.png; outputs/13_figures_diagrams/G10_feature_family_counts.csv; outputs/13_figures_diagrams/G10_feature_family_counts.meta.json; outputs/13_figures_diagrams/F02_end_to_end_pcg_classification_workflow.svg; outputs/13_figures_diagrams/F02_end_to_end_pcg_classification_workflow.png; outputs/13_figures_diagrams/F02_end_to_end_pcg_classification_workflow.meta.json; outputs/13_figures_diagrams/F04_dataset_harmonization_and_metadata_workflow.svg; outputs/13_figures_diagrams/F04_dataset_harmonization_and_metadata_workflow.png; outputs/13_figures_diagrams/F04_dataset_harmonization_and_metadata_workflow.meta.json; outputs/13_figures_diagrams/F05_subject_wise_data_splitting.svg; outputs/13_figures_diagrams/F05_subject_wise_data_splitting.png; outputs/13_figures_diagrams/F05_subject_wise_data_splitting.meta.json; outputs/13_figures_diagrams/F06_signal_preprocessing_architecture.svg; outputs/13_figures_diagrams/F06_signal_preprocessing_architecture.png; outputs/13_figures_diagrams/F06_signal_preprocessing_architecture.meta.json; outputs/13_figures_diagrams/F07_138_feature_extraction_architecture.svg; outputs/13_figures_diagrams/F07_138_feature_extraction_architecture.png; outputs/13_figures_diagrams/F07_138_feature_extraction_architecture.meta.json; outputs/13_figures_diagrams/F08_feature_family_fusion.svg; outputs/13_figures_diagrams/F08_feature_family_fusion.png; outputs/13_figures_diagrams/F08_feature_family_fusion.meta.json; outputs/13_figures_diagrams/F09_search_based_feature_selection_workflow.svg; outputs/13_figures_diagrams/F09_search_based_feature_selection_workflow.png; outputs/13_figures_diagrams/F09_search_based_feature_selection_workflow.meta.json; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.svg; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.png; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.meta.json; outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.docx; outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.txt; outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.docx; outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.txt; outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.docx; outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.txt; outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.docx; outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt; outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.docx; outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.txt; outputs/14_algorithms/ALG-06_search_based_feature_selection.docx; outputs/14_algorithms/ALG-06_search_based_feature_selection.txt; outputs/14_algorithms/ALG-07_hyperparameter_optimization.docx; outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt; outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.docx; outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.txt; outputs/14_algorithms/ALG-09_random_forest_training.docx; outputs/14_algorithms/ALG-09_random_forest_training.txt; outputs/14_algorithms/ALG-10_gradient_boosting_training.docx; outputs/14_algorithms/ALG-10_gradient_boosting_training.txt; outputs/14_algorithms/ALG-11_equal_weight_soft_voting.docx; outputs/14_algorithms/ALG-11_equal_weight_soft_voting.txt; outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.docx; outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt; outputs/14_algorithms/equations_reference.docx; outputs/14_algorithms/equations_reference.tex; outputs/14_algorithms/equations_reference.csv</t>
+        </is>
+      </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>python scripts/49_final_qa_sweep.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>2026-09-12T14:09:12.050185+00:00</t>
+          <t>2026-09-14T06:58:00.750638+00:00</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>no source_data recorded</t>
+          <t>file and 102 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>QA-COMPLIANCE</t>
-        </is>
-      </c>
-      <c r="B287" t="inlineStr"/>
+          <t>THESIS-Ch4_Implementation</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>O1-O6</t>
+        </is>
+      </c>
       <c r="C287" t="inlineStr"/>
       <c r="D287" t="inlineStr"/>
       <c r="E287" t="inlineStr"/>
       <c r="F287" t="inlineStr">
         <is>
-          <t>compliance and claims review (Phase 125)</t>
+          <t>Ch4_Implementation: 14 algorithm, 1 appendix, 21 diagram</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>outputs/00_evidence_index/compliance_review.md</t>
-        </is>
-      </c>
-      <c r="H287" t="inlineStr"/>
+          <t>outputs/THESIS_ASSETS/Ch4_Implementation/chapter_index.csv</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>outputs/13_figures_diagrams/F11_binary_classification_pipeline.svg; outputs/13_figures_diagrams/F11_binary_classification_pipeline.png; outputs/13_figures_diagrams/F11_binary_classification_pipeline.meta.json; outputs/13_figures_diagrams/F12_pascal_multiclass_pipeline.svg; outputs/13_figures_diagrams/F12_pascal_multiclass_pipeline.png; outputs/13_figures_diagrams/F12_pascal_multiclass_pipeline.meta.json; outputs/13_figures_diagrams/F13_circor_recording_to_subject_aggregation.svg; outputs/13_figures_diagrams/F13_circor_recording_to_subject_aggregation.png; outputs/13_figures_diagrams/F13_circor_recording_to_subject_aggregation.meta.json; outputs/13_figures_diagrams/F14_cross_dataset_external_validation_workflow.svg; outputs/13_figures_diagrams/F14_cross_dataset_external_validation_workflow.png; outputs/13_figures_diagrams/F14_cross_dataset_external_validation_workflow.meta.json; outputs/13_figures_diagrams/F15_noise_and_duration_robustness_framework.svg; outputs/13_figures_diagrams/F15_noise_and_duration_robustness_framework.png; outputs/13_figures_diagrams/F15_noise_and_duration_robustness_framework.meta.json; outputs/13_figures_diagrams/F16_dashboard_system_architecture.svg; outputs/13_figures_diagrams/F16_dashboard_system_architecture.png; outputs/13_figures_diagrams/F16_dashboard_system_architecture.meta.json; outputs/13_figures_diagrams/F17_prediction_and_report_generation_flow.svg; outputs/13_figures_diagrams/F17_prediction_and_report_generation_flow.png; outputs/13_figures_diagrams/F17_prediction_and_report_generation_flow.meta.json; outputs/14_algorithms/ALG-13_binary_evaluation_workflow.docx; outputs/14_algorithms/ALG-13_binary_evaluation_workflow.txt; outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.docx; outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.txt; outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.docx; outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.txt; outputs/14_algorithms/ALG-16_cross_dataset_external_validation.docx; outputs/14_algorithms/ALG-16_cross_dataset_external_validation.txt; outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.docx; outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.txt; outputs/14_algorithms/ALG-18_failure_case_analysis.docx; outputs/14_algorithms/ALG-18_failure_case_analysis.txt; outputs/14_algorithms/ALG-19_sample_level_report_generation.docx; outputs/14_algorithms/ALG-19_sample_level_report_generation.txt; outputs/00_evidence_index/run_manifest.json; outputs/00_evidence_index/evidence_index.csv</t>
+        </is>
+      </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>python scripts/50_compliance_review.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>2026-09-12T14:10:21.244861+00:00</t>
+          <t>2026-09-14T06:58:00.850122+00:00</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>no source_data recorded</t>
+          <t>file and 37 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>DOC-ARCH</t>
-        </is>
-      </c>
-      <c r="B288" t="inlineStr"/>
+          <t>THESIS-Ch5_Results</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>O1-O6</t>
+        </is>
+      </c>
       <c r="C288" t="inlineStr"/>
       <c r="D288" t="inlineStr"/>
       <c r="E288" t="inlineStr"/>
       <c r="F288" t="inlineStr">
         <is>
-          <t>project structure and the role of each module (T123.2)</t>
+          <t>Ch5_Results: 75 graph, 63 table</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>ARCHITECTURE.md</t>
-        </is>
-      </c>
-      <c r="H288" t="inlineStr"/>
+          <t>outputs/THESIS_ASSETS/Ch5_Results/chapter_index.csv</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>outputs/06_binary_results/T08_physionet_individual_model_comparison.csv; outputs/06_binary_results/T08_physionet_individual_model_comparison.docx; outputs/06_binary_results/T08_physionet_individual_model_comparison.meta.json; outputs/06_binary_results/T09_equal_weight_versus_optimized_ensemble.csv; outputs/06_binary_results/T09_equal_weight_versus_optimized_ensemble.docx; outputs/06_binary_results/T09_equal_weight_versus_optimized_ensemble.meta.json; outputs/06_binary_results/T10_physionet_fold_wise_results.csv; outputs/06_binary_results/T10_physionet_fold_wise_results.docx; outputs/06_binary_results/T10_physionet_fold_wise_results.meta.json; outputs/07_multiclass_results/T11_pascal_a_multiclass_results.csv; outputs/07_multiclass_results/T11_pascal_a_multiclass_results.docx; outputs/07_multiclass_results/T11_pascal_a_multiclass_results.meta.json; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.csv; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.docx; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.meta.json; outputs/08_circor_external_validation/T13_circor_murmur_classification_results.csv; outputs/08_circor_external_validation/T13_circor_murmur_classification_results.docx; outputs/08_circor_external_validation/T13_circor_murmur_classification_results.meta.json; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.csv; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.docx; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.meta.json; outputs/08_circor_external_validation/T15_recording_level_versus_subject_level_results.csv; outputs/08_circor_external_validation/T15_recording_level_versus_subject_level_results.docx; outputs/08_circor_external_validation/T15_recording_level_versus_subject_level_results.meta.json; outputs/08_circor_external_validation/T16_cross_dataset_generalization.csv; outputs/08_circor_external_validation/T16_cross_dataset_generalization.docx; outputs/08_circor_external_validation/T16_cross_dataset_generalization.meta.json; outputs/09_ablation/T17_feature_family_ablation.csv; outputs/09_ablation/T17_feature_family_ablation.docx; outputs/09_ablation/T17_feature_family_ablation.meta.json; outputs/09_ablation/T18_all_features_versus_selected_features.csv; outputs/09_ablation/T18_all_features_versus_selected_features.docx; outputs/09_ablation/T18_all_features_versus_selected_features.meta.json; outputs/09_ablation/T19_search_and_optimization_ablation.csv; outputs/09_ablation/T19_search_and_optimization_ablation.docx; outputs/09_ablation/T19_search_and_optimization_ablation.meta.json; outputs/09_robustness_analysis/T20_noise_robustness.csv; outputs/09_robustness_analysis/T20_noise_robustness.docx; outputs/09_robustness_analysis/T20_noise_robustness.meta.json; outputs/09_robustness_analysis/T21_duration_robustness.csv; outputs/09_robustness_analysis/T21_duration_robustness.docx; outputs/09_robustness_analysis/T21_duration_robustness.meta.json; outputs/08_circor_external_validation/T22_auscultation_location_analysis.csv; outputs/08_circor_external_validation/T22_auscultation_location_analysis.docx; outputs/08_circor_external_validation/T22_auscultation_location_analysis.meta.json; outputs/10_robustness/T23_calibration_and_confidence_summary.csv; outputs/10_robustness/T23_calibration_and_confidence_summary.docx; outputs/10_robustness/T23_calibration_and_confidence_summary.meta.json; outputs/11_complexity/T24_complexity_analysis.csv; outputs/11_complexity/T24_complexity_analysis.docx; outputs/11_complexity/T24_complexity_analysis.meta.json; outputs/11_complexity/T25_training_and_inference_time.csv; outputs/11_complexity/T25_training_and_inference_time.docx; outputs/11_complexity/T25_training_and_inference_time.meta.json; outputs/11_complexity/T26_model_size_and_memory.csv; outputs/11_complexity/T26_model_size_and_memory.docx; outputs/11_complexity/T26_model_size_and_memory.meta.json; outputs/10_robustness/T27_false_positive_and_false_negative_analysis.csv; outputs/10_robustness/T27_false_positive_and_false_negative_analysis.docx; outputs/10_robustness/T27_false_positive_and_false_negative_analysis.meta.json; outputs/12_statistics/T28_statistical_significance_comparison.csv; outputs/12_statistics/T28_statistical_significance_comparison.docx; outputs/12_statistics/T28_statistical_significance_comparison.meta.json; outputs/13_figures_diagrams/G11_individual_model_comparison.png; outputs/13_figures_diagrams/G11_individual_model_comparison.csv; outputs/13_figures_diagrams/G11_individual_model_comparison.meta.json; outputs/13_figures_diagrams/G12_binary_roc_curve.png; outputs/13_figures_diagrams/G12_binary_roc_curve.csv; outputs/13_figures_diagrams/G12_binary_roc_curve.meta.json; outputs/13_figures_diagrams/G13_binary_precision_recall_curve.png; outputs/13_figures_diagrams/G13_binary_precision_recall_curve.csv; outputs/13_figures_diagrams/G13_binary_precision_recall_curve.meta.json; outputs/13_figures_diagrams/G14_binary_confusion_matrix.png; outputs/13_figures_diagrams/G14_binary_confusion_matrix.csv; outputs/13_figures_diagrams/G14_binary_confusion_matrix.meta.json; outputs/13_figures_diagrams/G15_pascal_a_confusion_matrix.png; outputs/13_figures_diagrams/G15_pascal_a_confusion_matrix.csv; outputs/13_figures_diagrams/G15_pascal_a_confusion_matrix.meta.json; outputs/13_figures_diagrams/G16_pascal_b_confusion_matrix.png; outputs/13_figures_diagrams/G16_pascal_b_confusion_matrix.csv; outputs/13_figures_diagrams/G16_pascal_b_confusion_matrix.meta.json; outputs/13_figures_diagrams/G17_multiclass_one_vs_rest_roc.png; outputs/13_figures_diagrams/G17_multiclass_one_vs_rest_roc.csv; outputs/13_figures_diagrams/G17_multiclass_one_vs_rest_roc.meta.json; outputs/13_figures_diagrams/G18_feature_importance_plot.png; outputs/13_figures_diagrams/G18_feature_importance_plot.csv; outputs/13_figures_diagrams/G18_feature_importance_plot.meta.json; outputs/13_figures_diagrams/G19_top_20_features_chart.png; outputs/13_figures_diagrams/G19_top_20_features_chart.csv; outputs/13_figures_diagrams/G19_top_20_features_chart.meta.json; outputs/13_figures_diagrams/G20_search_convergence_plot.png; outputs/13_figures_diagrams/G20_search_convergence_plot.csv; outputs/13_figures_diagrams/G20_search_convergence_plot.meta.json; outputs/13_figures_diagrams/G21_all_features_versus_selected_features.png; outputs/13_figures_diagrams/G21_all_features_versus_selected_features.csv; outputs/13_figures_diagrams/G21_all_features_versus_selected_features.meta.json; outputs/13_figures_diagrams/G22_f1_and_accuracy_versus_feature_count.png; outputs/13_figures_diagrams/G22_f1_and_accuracy_versus_feature_count.csv; outputs/13_figures_diagrams/G22_f1_and_accuracy_versus_feature_count.meta.json; outputs/13_figures_diagrams/G23_ensemble_weight_comparison.png; outputs/13_figures_diagrams/G23_ensemble_weight_comparison.csv; outputs/13_figures_diagrams/G23_ensemble_weight_comparison.meta.json; outputs/13_figures_diagrams/G24_baseline_versus_optimized.png; outputs/13_figures_diagrams/G24_baseline_versus_optimized.csv; outputs/13_figures_diagrams/G24_baseline_versus_optimized.meta.json; outputs/13_figures_diagrams/G25_inference_time_versus_performance.png; outputs/13_figures_diagrams/G25_inference_time_versus_performance.csv; outputs/13_figures_diagrams/G25_inference_time_versus_performance.meta.json; outputs/13_figures_diagrams/G26_training_time_comparison.png; outputs/13_figures_diagrams/G26_training_time_comparison.csv; outputs/13_figures_diagrams/G26_training_time_comparison.meta.json; outputs/13_figures_diagrams/G27_model_size_comparison.png; outputs/13_figures_diagrams/G27_model_size_comparison.csv; outputs/13_figures_diagrams/G27_model_size_comparison.meta.json; outputs/13_figures_diagrams/G28_dataset_wise_generalization.png; outputs/13_figures_diagrams/G28_dataset_wise_generalization.csv; outputs/13_figures_diagrams/G28_dataset_wise_generalization.meta.json; outputs/13_figures_diagrams/G29_cross_dataset_performance_drop.png; outputs/13_figures_diagrams/G29_cross_dataset_performance_drop.csv; outputs/13_figures_diagrams/G29_cross_dataset_performance_drop.meta.json; outputs/13_figures_diagrams/G30_noise_level_robustness.png; outputs/13_figures_diagrams/G30_noise_level_robustness.csv; outputs/13_figures_diagrams/G30_noise_level_robustness.meta.json; outputs/13_figures_diagrams/G31_duration_wise_performance.png; outputs/13_figures_diagrams/G31_duration_wise_performance.csv; outputs/13_figures_diagrams/G31_duration_wise_performance.meta.json; outputs/13_figures_diagrams/G32_location_performance.png; outputs/13_figures_diagrams/G32_location_performance.csv; outputs/13_figures_diagrams/G32_location_performance.meta.json; outputs/13_figures_diagrams/G33_confidence_histogram.png; outputs/13_figures_diagrams/G33_confidence_histogram.csv; outputs/13_figures_diagrams/G33_confidence_histogram.meta.json; outputs/13_figures_diagrams/G34_calibration_curve.png; outputs/13_figures_diagrams/G34_calibration_curve.csv; outputs/13_figures_diagrams/G34_calibration_curve.meta.json; outputs/13_figures_diagrams/G35_false_positive_and_false_negative_distribution.png; outputs/13_figures_diagrams/G35_false_positive_and_false_negative_distribution.csv; outputs/13_figures_diagrams/G35_false_positive_and_false_negative_distribution.meta.json</t>
+        </is>
+      </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>python scripts/48_project_docs.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>2026-09-12T15:31:30.904931+00:00</t>
+          <t>2026-09-14T06:58:00.968036+00:00</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>no source_data recorded</t>
+          <t>file and 138 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>DOC-CONFIG</t>
-        </is>
-      </c>
-      <c r="B289" t="inlineStr"/>
+          <t>THESIS-Ch6_Conclusion</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>O1-O6</t>
+        </is>
+      </c>
       <c r="C289" t="inlineStr"/>
       <c r="D289" t="inlineStr"/>
       <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
         <is>
-          <t>every configuration option and its default (T123.3)</t>
+          <t>Ch6_Conclusion: 2 algorithm, 6 diagram, 6 table</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>CONFIGURATION.md</t>
+          <t>outputs/THESIS_ASSETS/Ch6_Conclusion/chapter_index.csv</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>configs</t>
+          <t>outputs/00_evidence_index/T29_objective_to_evidence_mapping.csv; outputs/00_evidence_index/T29_objective_to_evidence_mapping.docx; outputs/00_evidence_index/T29_objective_to_evidence_mapping.meta.json; outputs/00_evidence_index/T30_final_conclusion_matrix.csv; outputs/00_evidence_index/T30_final_conclusion_matrix.docx; outputs/00_evidence_index/T30_final_conclusion_matrix.meta.json; outputs/13_figures_diagrams/F18_objective_to_module_traceability.svg; outputs/13_figures_diagrams/F18_objective_to_module_traceability.png; outputs/13_figures_diagrams/F18_objective_to_module_traceability.meta.json; outputs/13_figures_diagrams/F20_final_research_contribution_summary.svg; outputs/13_figures_diagrams/F20_final_research_contribution_summary.png; outputs/13_figures_diagrams/F20_final_research_contribution_summary.meta.json; outputs/14_algorithms/ALG-20_objective_achievement_evidence_generation.docx; outputs/14_algorithms/ALG-20_objective_achievement_evidence_generation.txt</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>python scripts/48_project_docs.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>2026-09-12T15:31:31.056618+00:00</t>
+          <t>2026-09-14T06:58:00.998820+00:00</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -15606,14 +15602,14 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>file on disk; source is descriptive, not a path</t>
+          <t>file and 14 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>DOC-HANDOVER</t>
+          <t>THESIS-REPRODUCIBILITY</t>
         </is>
       </c>
       <c r="B290" t="inlineStr"/>
@@ -15622,33 +15618,37 @@
       <c r="E290" t="inlineStr"/>
       <c r="F290" t="inlineStr">
         <is>
-          <t>handover summary: produced, not produced, next steps (T126.6)</t>
+          <t>reproducibility appendix: environment, seeds, packages, stage timing, commands</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>HANDOVER.md</t>
-        </is>
-      </c>
-      <c r="H290" t="inlineStr"/>
+          <t>outputs/THESIS_ASSETS/Ch4_Implementation/reproducibility_appendix.docx</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>outputs/00_evidence_index/run_manifest.json</t>
+        </is>
+      </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>python scripts/51_package_delivery.py</t>
+          <t>python scripts/44_thesis_assets.py</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>2026-09-12T15:32:49.621460+00:00</t>
+          <t>2026-09-14T06:58:01.026013+00:00</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>no source_data recorded</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
@@ -27668,7 +27668,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-13T17:10:22.966579+00:00</t>
+          <t>2026-09-14T06:58:03.620289+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 131: Analyse batch and compare -- batch mode with per-file progress, skip and cancel, sortable table with outcome counts, one batch id per batch in History, side-by-side compare view, refused files kept as rows, CSV written server-side from History
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/00_evidence_index/evidence_index.xlsx
+++ b/outputs/00_evidence_index/evidence_index.xlsx
@@ -15292,7 +15292,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>2026-09-14T06:57:31.724955+00:00</t>
+          <t>2026-09-14T11:29:46.444033+00:00</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -15342,7 +15342,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:00.652545+00:00</t>
+          <t>2026-09-14T11:31:53.025203+00:00</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -15392,7 +15392,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:00.667352+00:00</t>
+          <t>2026-09-14T11:31:53.088963+00:00</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -15442,7 +15442,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:00.750638+00:00</t>
+          <t>2026-09-14T11:31:53.308687+00:00</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -15492,7 +15492,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:00.850122+00:00</t>
+          <t>2026-09-14T11:31:53.427137+00:00</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -15542,7 +15542,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:00.968036+00:00</t>
+          <t>2026-09-14T11:31:53.657298+00:00</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -15592,7 +15592,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:00.998820+00:00</t>
+          <t>2026-09-14T11:31:53.750411+00:00</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -15638,7 +15638,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>2026-09-14T06:58:01.026013+00:00</t>
+          <t>2026-09-14T11:31:53.825130+00:00</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -27668,7 +27668,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-14T10:25:40.447604+00:00</t>
+          <t>2026-09-14T11:44:11.237332+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 132: History page -- server-filtered list with search, result/task/tag/date filters kept in the address, record drawer with waveform for sample entries and notes/tags editing, delete with undo (restore route) and delete-all with confirmation, compare two records, fresh-install empty state
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/00_evidence_index/evidence_index.xlsx
+++ b/outputs/00_evidence_index/evidence_index.xlsx
@@ -15292,7 +15292,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>2026-09-14T11:29:46.444033+00:00</t>
+          <t>2026-09-14T12:21:44.334339+00:00</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -15342,7 +15342,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.025203+00:00</t>
+          <t>2026-09-14T12:21:53.072844+00:00</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -15392,7 +15392,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.088963+00:00</t>
+          <t>2026-09-14T12:21:53.101599+00:00</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -15442,7 +15442,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.308687+00:00</t>
+          <t>2026-09-14T12:21:53.171982+00:00</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -15492,7 +15492,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.427137+00:00</t>
+          <t>2026-09-14T12:21:53.201288+00:00</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -15542,7 +15542,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.657298+00:00</t>
+          <t>2026-09-14T12:21:53.273337+00:00</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -15592,7 +15592,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.750411+00:00</t>
+          <t>2026-09-14T12:21:53.303130+00:00</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -15638,7 +15638,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>2026-09-14T11:31:53.825130+00:00</t>
+          <t>2026-09-14T12:21:53.319235+00:00</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -27668,7 +27668,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-14T11:44:11.237332+00:00</t>
+          <t>2026-09-14T12:54:37.603884+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>